<commit_message>
Guía paso a paso parte 1 y tabla de variables Rev. B
- Tabla Rev. B: decisiones confirmadas, I0.7 SW_Prueba_Nivel_99
- Fuentes externas de UDT_Botella, DB_Linea, DB_FIFO y DB_Tiempos
- Guía: proyecto, hardware, importación de variables, DBs, OB30,
  OB100 y FC1 en KOP, con prueba en PLCSIM
- Dibujo de segmentos KOP en texto generado (herramientas/kop.py)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LWd5edd3sJ42yUMBzfU6c6
</commit_message>
<xml_diff>
--- a/tia/Variables_PLC.xlsx
+++ b/tia/Variables_PLC.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -796,7 +796,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>S_Botella_Bajo</t>
+          <t>SW_Prueba_Nivel_99</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -811,12 +811,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>%I1.0</t>
+          <t>%I0.7</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sensor altura BAJA (detecta cualquier botella)</t>
+          <t>Interruptor PRUEBAS: bomba no para al 90 %</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -840,7 +840,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>S_Botella_Alto</t>
+          <t>S_Botella_Bajo</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>%I1.1</t>
+          <t>%I1.0</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sensor altura ALTA (solo botella 2 L)</t>
+          <t>Sensor altura BAJA (detecta cualquier botella)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -884,7 +884,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>S_Pos_Llenado</t>
+          <t>S_Botella_Alto</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -899,12 +899,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>%I1.2</t>
+          <t>%I1.1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Botella en posición de LLENADO</t>
+          <t>Sensor altura ALTA (solo botella 2 L)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -928,7 +928,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>S_Pos_Taponado</t>
+          <t>S_Pos_Llenado</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -943,12 +943,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>%I1.3</t>
+          <t>%I1.2</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Botella en posición TAP-01</t>
+          <t>Botella en posición de LLENADO</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -972,7 +972,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>S_Pos_Rechazo</t>
+          <t>S_Pos_Taponado</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -987,12 +987,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>%I1.4</t>
+          <t>%I1.3</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Botella frente al EMPUJADOR</t>
+          <t>Botella en posición TAP-01</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1016,7 +1016,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>S_Entrada_Transversal</t>
+          <t>S_Pos_Rechazo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1031,12 +1031,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>%I1.5</t>
+          <t>%I1.4</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Botella entra en cinta transversal C5</t>
+          <t>Botella frente al EMPUJADOR</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1060,7 +1060,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>S_TAP01_Arriba</t>
+          <t>S_Entrada_Transversal</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>%I2.0</t>
+          <t>%I1.5</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>TAP-01 cabezal ARRIBA</t>
+          <t>Botella entra en cinta transversal C5</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1104,7 +1104,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>S_TAP01_Abajo</t>
+          <t>S_TAP01_Arriba</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1119,12 +1119,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>%I2.1</t>
+          <t>%I2.0</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>TAP-01 cabezal ABAJO (tapón puesto)</t>
+          <t>TAP-01 cabezal ARRIBA</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1148,7 +1148,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>S_Empujador_Atras</t>
+          <t>S_TAP01_Abajo</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1163,12 +1163,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>%I2.2</t>
+          <t>%I2.1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Empujador RETROCEDIDO</t>
+          <t>TAP-01 cabezal ABAJO (tapón puesto)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1192,7 +1192,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>S_Empujador_Delante</t>
+          <t>S_Empujador_Atras</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1207,12 +1207,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>%I2.3</t>
+          <t>%I2.2</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Empujador AVANZADO</t>
+          <t>Empujador RETROCEDIDO</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1236,7 +1236,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>S_Caja_Malas_Entrada</t>
+          <t>S_Empujador_Delante</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1251,12 +1251,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>%I2.4</t>
+          <t>%I2.3</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Botella cae en caja MALAS</t>
+          <t>Empujador AVANZADO</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1280,7 +1280,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>S_Caja_05L_Entrada</t>
+          <t>S_Caja_Malas_Entrada</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1295,12 +1295,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>%I2.5</t>
+          <t>%I2.4</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Botella cae en caja 0,5 L</t>
+          <t>Botella cae en caja MALAS</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1324,7 +1324,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>S_Caja_2L_Entrada</t>
+          <t>S_Caja_05L_Entrada</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1339,12 +1339,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>%I2.6</t>
+          <t>%I2.5</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Botella cae en caja 2 L</t>
+          <t>Botella cae en caja 0,5 L</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1368,7 +1368,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>S_Caja_Malas_Presente</t>
+          <t>S_Caja_2L_Entrada</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1383,12 +1383,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>%I3.0</t>
+          <t>%I2.6</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Caja de MALAS en su sitio</t>
+          <t>Botella cae en caja 2 L</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1412,7 +1412,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>S_Caja_05L_Presente</t>
+          <t>S_Caja_Malas_Presente</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1427,12 +1427,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>%I3.1</t>
+          <t>%I3.0</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Caja de 0,5 L en su sitio</t>
+          <t>Caja de MALAS en su sitio</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>S_Caja_2L_Presente</t>
+          <t>S_Caja_05L_Presente</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1471,12 +1471,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>%I3.2</t>
+          <t>%I3.1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Caja de 2 L en su sitio</t>
+          <t>Caja de 0,5 L en su sitio</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1500,7 +1500,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>S_Tanque_25</t>
+          <t>S_Caja_2L_Presente</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>%I3.3</t>
+          <t>%I3.2</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Sensor nivel tanque 25 % (instalación real)</t>
+          <t>Caja de 2 L en su sitio</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1544,7 +1544,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>S_Tanque_90</t>
+          <t>S_Tanque_25</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1559,12 +1559,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>%I3.4</t>
+          <t>%I3.3</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Sensor nivel tanque 90 % (instalación real)</t>
+          <t>Sensor nivel tanque 25 % (instalación real)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1588,7 +1588,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>S_Tanque_99</t>
+          <t>S_Tanque_90</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1603,12 +1603,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>%I3.5</t>
+          <t>%I3.4</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Sensor nivel tanque 99 % (instalación real)</t>
+          <t>Sensor nivel tanque 90 % (instalación real)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1632,7 +1632,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>VS_Valvula_Seguridad</t>
+          <t>S_Tanque_99</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>%Q0.0</t>
+          <t>%I3.5</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Válvula de seguridad tanque · 1 = ABIERTA</t>
+          <t>Sensor nivel tanque 99 % (instalación real)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1676,7 +1676,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Baliza_Naranja</t>
+          <t>VS_Valvula_Seguridad</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1691,12 +1691,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>%Q0.1</t>
+          <t>%Q0.0</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Baliza naranja de emergencia (intermitente)</t>
+          <t>Válvula de seguridad tanque · 1 = ABIERTA</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1720,7 +1720,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sirena</t>
+          <t>Baliza_Naranja</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1735,12 +1735,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>%Q0.2</t>
+          <t>%Q0.1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Sirena de emergencia</t>
+          <t>Baliza naranja de emergencia (intermitente)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1764,7 +1764,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Emisor_Botellas</t>
+          <t>Sirena</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1779,12 +1779,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>%Q0.3</t>
+          <t>%Q0.2</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Generador de botellas (pulso = 1 botella)</t>
+          <t>Sirena de emergencia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1808,7 +1808,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cinta_C1_Entrada</t>
+          <t>Emisor_Botellas</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1823,12 +1823,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>%Q0.4</t>
+          <t>%Q0.3</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Cinta C1: generador → detección</t>
+          <t>Generador de botellas (pulso = 1 botella)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1852,7 +1852,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cinta_C2_Llenado</t>
+          <t>Cinta_C1_Entrada</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1867,12 +1867,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>%Q0.5</t>
+          <t>%Q0.4</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Cinta C2: zona de llenado</t>
+          <t>Cinta C1: generador → detección</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1896,7 +1896,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Cinta_C3_Taponado</t>
+          <t>Cinta_C2_Llenado</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1911,12 +1911,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>%Q0.6</t>
+          <t>%Q0.5</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Cinta C3: zona TAP-01</t>
+          <t>Cinta C2: zona de llenado</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1940,7 +1940,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cinta_C4_Rechazo</t>
+          <t>Cinta_C3_Taponado</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1955,12 +1955,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>%Q0.7</t>
+          <t>%Q0.6</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Cinta C4: zona empujador</t>
+          <t>Cinta C3: zona TAP-01</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1984,7 +1984,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cinta_C5_Hacia_05L</t>
+          <t>Cinta_C4_Rechazo</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1999,12 +1999,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>%Q1.0</t>
+          <t>%Q0.7</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Cinta transversal C5 → caja 0,5 L</t>
+          <t>Cinta C4: zona empujador</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2028,7 +2028,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cinta_C5_Hacia_2L</t>
+          <t>Cinta_C5_Hacia_05L</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2043,12 +2043,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>%Q1.1</t>
+          <t>%Q1.0</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Cinta transversal C5 → caja 2 L</t>
+          <t>Cinta transversal C5 → caja 0,5 L</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2072,7 +2072,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TAP01_Bajar</t>
+          <t>Cinta_C5_Hacia_2L</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2087,12 +2087,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>%Q2.0</t>
+          <t>%Q1.1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>TAP-01 bajar cabezal</t>
+          <t>Cinta transversal C5 → caja 2 L</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2116,7 +2116,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Empujador_Avanzar</t>
+          <t>TAP01_Bajar</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2131,12 +2131,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>%Q2.1</t>
+          <t>%Q2.0</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Empujador botellas malas: avanzar</t>
+          <t>TAP-01 bajar cabezal</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2160,7 +2160,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Caja_Malas_Retirar</t>
+          <t>Empujador_Avanzar</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2175,12 +2175,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>%Q2.2</t>
+          <t>%Q2.1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Retirar caja MALAS (llena)</t>
+          <t>Empujador botellas malas: avanzar</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2204,7 +2204,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Caja_Malas_Reponer</t>
+          <t>Caja_Malas_Retirar</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2219,12 +2219,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>%Q2.3</t>
+          <t>%Q2.2</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Poner caja MALAS nueva</t>
+          <t>Retirar caja MALAS (llena)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2248,7 +2248,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Caja_05L_Retirar</t>
+          <t>Caja_Malas_Reponer</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2263,12 +2263,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>%Q2.4</t>
+          <t>%Q2.3</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Retirar caja 0,5 L (llena)</t>
+          <t>Poner caja MALAS nueva</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2292,7 +2292,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Caja_05L_Reponer</t>
+          <t>Caja_05L_Retirar</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2307,12 +2307,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>%Q2.5</t>
+          <t>%Q2.4</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Poner caja 0,5 L nueva</t>
+          <t>Retirar caja 0,5 L (llena)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2336,7 +2336,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Caja_2L_Retirar</t>
+          <t>Caja_05L_Reponer</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2351,12 +2351,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>%Q2.6</t>
+          <t>%Q2.5</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Retirar caja 2 L (llena)</t>
+          <t>Poner caja 0,5 L nueva</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2380,7 +2380,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Caja_2L_Reponer</t>
+          <t>Caja_2L_Retirar</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2395,12 +2395,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>%Q2.7</t>
+          <t>%Q2.6</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Poner caja 2 L nueva</t>
+          <t>Retirar caja 2 L (llena)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Piloto_Marcha</t>
+          <t>Caja_2L_Reponer</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2439,12 +2439,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>%Q3.0</t>
+          <t>%Q2.7</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Piloto verde MARCHA</t>
+          <t>Poner caja 2 L nueva</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2468,7 +2468,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Piloto_Paro</t>
+          <t>Piloto_Marcha</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2483,12 +2483,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>%Q3.1</t>
+          <t>%Q3.0</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Piloto rojo PARO</t>
+          <t>Piloto verde MARCHA</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2512,7 +2512,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Piloto_Rearme</t>
+          <t>Piloto_Paro</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2527,12 +2527,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>%Q3.2</t>
+          <t>%Q3.1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Piloto azul REARME</t>
+          <t>Piloto rojo PARO</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2556,7 +2556,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>L1_Tanque_Verde</t>
+          <t>Piloto_Rearme</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2571,12 +2571,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>%Q3.3</t>
+          <t>%Q3.2</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Fase 1 Tanque · lámpara verde</t>
+          <t>Piloto azul REARME</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2600,7 +2600,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>L1_Tanque_Naranja</t>
+          <t>L1_Tanque_Verde</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2615,12 +2615,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>%Q3.4</t>
+          <t>%Q3.3</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Fase 1 Tanque · lámpara naranja</t>
+          <t>Fase 1 Tanque · lámpara verde</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2644,7 +2644,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>L1_Tanque_Rojo</t>
+          <t>L1_Tanque_Naranja</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2659,12 +2659,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>%Q3.5</t>
+          <t>%Q3.4</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Fase 1 Tanque · lámpara roja</t>
+          <t>Fase 1 Tanque · lámpara naranja</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2688,7 +2688,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>L2_Deteccion_Verde</t>
+          <t>L1_Tanque_Rojo</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2703,12 +2703,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>%Q3.6</t>
+          <t>%Q3.5</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Fase 2 Generación y detección · lámpara verde</t>
+          <t>Fase 1 Tanque · lámpara roja</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2732,7 +2732,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>L2_Deteccion_Naranja</t>
+          <t>L2_Deteccion_Verde</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2747,12 +2747,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>%Q3.7</t>
+          <t>%Q3.6</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Fase 2 Generación y detección · lámpara naranja</t>
+          <t>Fase 2 Generación y detección · lámpara verde</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2776,7 +2776,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>L2_Deteccion_Rojo</t>
+          <t>L2_Deteccion_Naranja</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2791,12 +2791,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>%Q4.0</t>
+          <t>%Q3.7</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Fase 2 Generación y detección · lámpara roja</t>
+          <t>Fase 2 Generación y detección · lámpara naranja</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2820,7 +2820,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>L3_Llenado_Verde</t>
+          <t>L2_Deteccion_Rojo</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2835,12 +2835,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>%Q4.1</t>
+          <t>%Q4.0</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Fase 3 Llenado · lámpara verde</t>
+          <t>Fase 2 Generación y detección · lámpara roja</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2864,7 +2864,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>L3_Llenado_Naranja</t>
+          <t>L3_Llenado_Verde</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2879,12 +2879,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>%Q4.2</t>
+          <t>%Q4.1</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Fase 3 Llenado · lámpara naranja</t>
+          <t>Fase 3 Llenado · lámpara verde</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2908,7 +2908,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>L3_Llenado_Rojo</t>
+          <t>L3_Llenado_Naranja</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2923,12 +2923,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>%Q4.3</t>
+          <t>%Q4.2</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Fase 3 Llenado · lámpara roja</t>
+          <t>Fase 3 Llenado · lámpara naranja</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2952,7 +2952,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>L4_Taponado_Verde</t>
+          <t>L3_Llenado_Rojo</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2967,12 +2967,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>%Q4.4</t>
+          <t>%Q4.3</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Fase 4 Taponado TAP-01 · lámpara verde</t>
+          <t>Fase 3 Llenado · lámpara roja</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2996,7 +2996,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>L4_Taponado_Naranja</t>
+          <t>L4_Taponado_Verde</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3011,12 +3011,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>%Q4.5</t>
+          <t>%Q4.4</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Fase 4 Taponado TAP-01 · lámpara naranja</t>
+          <t>Fase 4 Taponado TAP-01 · lámpara verde</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3040,7 +3040,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>L4_Taponado_Rojo</t>
+          <t>L4_Taponado_Naranja</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3055,12 +3055,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>%Q4.6</t>
+          <t>%Q4.5</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Fase 4 Taponado TAP-01 · lámpara roja</t>
+          <t>Fase 4 Taponado TAP-01 · lámpara naranja</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3084,7 +3084,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>L5_Rechazo_Verde</t>
+          <t>L4_Taponado_Rojo</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3099,12 +3099,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>%Q4.7</t>
+          <t>%Q4.6</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Fase 5 Rechazo de malas · lámpara verde</t>
+          <t>Fase 4 Taponado TAP-01 · lámpara roja</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3128,7 +3128,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>L5_Rechazo_Naranja</t>
+          <t>L5_Rechazo_Verde</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3143,12 +3143,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>%Q5.0</t>
+          <t>%Q4.7</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Fase 5 Rechazo de malas · lámpara naranja</t>
+          <t>Fase 5 Rechazo de malas · lámpara verde</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3172,7 +3172,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>L5_Rechazo_Rojo</t>
+          <t>L5_Rechazo_Naranja</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3187,12 +3187,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>%Q5.1</t>
+          <t>%Q5.0</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Fase 5 Rechazo de malas · lámpara roja</t>
+          <t>Fase 5 Rechazo de malas · lámpara naranja</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3216,7 +3216,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>L6_Clasif_Verde</t>
+          <t>L5_Rechazo_Rojo</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3231,12 +3231,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>%Q5.2</t>
+          <t>%Q5.1</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Fase 6 Clasificación y cajas · lámpara verde</t>
+          <t>Fase 5 Rechazo de malas · lámpara roja</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3260,7 +3260,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>L6_Clasif_Naranja</t>
+          <t>L6_Clasif_Verde</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3275,12 +3275,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>%Q5.3</t>
+          <t>%Q5.2</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Fase 6 Clasificación y cajas · lámpara naranja</t>
+          <t>Fase 6 Clasificación y cajas · lámpara verde</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3304,7 +3304,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>L6_Clasif_Rojo</t>
+          <t>L6_Clasif_Naranja</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3319,12 +3319,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>%Q5.4</t>
+          <t>%Q5.3</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Fase 6 Clasificación y cajas · lámpara roja</t>
+          <t>Fase 6 Clasificación y cajas · lámpara naranja</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3348,7 +3348,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>L7_General_Verde</t>
+          <t>L6_Clasif_Rojo</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3363,12 +3363,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>%Q5.5</t>
+          <t>%Q5.4</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Fase 7 General de línea · lámpara verde</t>
+          <t>Fase 6 Clasificación y cajas · lámpara roja</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3392,7 +3392,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>L7_General_Naranja</t>
+          <t>L7_General_Verde</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3407,12 +3407,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>%Q5.6</t>
+          <t>%Q5.5</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Fase 7 General de línea · lámpara naranja</t>
+          <t>Fase 7 General de línea · lámpara verde</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3436,7 +3436,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>L7_General_Rojo</t>
+          <t>L7_General_Naranja</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3451,12 +3451,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>%Q5.7</t>
+          <t>%Q5.6</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Fase 7 General de línea · lámpara roja</t>
+          <t>Fase 7 General de línea · lámpara naranja</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3480,7 +3480,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>AI_Nivel_Tanque</t>
+          <t>L7_General_Rojo</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3490,17 +3490,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Int</t>
+          <t>Bool</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>%IW64</t>
+          <t>%Q5.7</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Nivel tanque 0–27648 = 0–100 %</t>
+          <t>Fase 7 General de línea · lámpara roja</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3524,7 +3524,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>AI_Caudalimetro</t>
+          <t>AI_Nivel_Tanque</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3539,12 +3539,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>%IW66</t>
+          <t>%IW64</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Caudalímetro 0–27648 = 0–Caudal_Max l/min</t>
+          <t>Nivel tanque 0–27648 = 0–100 %</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3568,7 +3568,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>AQ_Bomba_Tanque</t>
+          <t>AI_Caudalimetro</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3583,12 +3583,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>%QW64</t>
+          <t>%IW66</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Bomba tanque · 27648 = 100 %, 0 = parada</t>
+          <t>Caudalímetro 0–27648 = 0–Caudal_Max l/min</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3612,7 +3612,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>AQ_Valvula_Llenado</t>
+          <t>AQ_Bomba_Tanque</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3627,12 +3627,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>%QW66</t>
+          <t>%QW64</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Válvula llenado botellas · 0 = cerrada</t>
+          <t>Bomba tanque · 27648 = 100 %, 0 = parada</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3652,6 +3652,50 @@
       </c>
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>AQ_Valvula_Llenado</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Linea_Llenado</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Int</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>%QW66</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Válvula llenado botellas · 0 = cerrada</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>